<commit_message>
fixture: Oznur PDF cevriminde buyuk X kabul ediliyor
Erce'nin duzeltmesi. Kesit ifadesi PDF'te bazen '4X25' seklinde buyuk harfle
geciyordu; regex yalnizca kucuk x kabul ediyordu. Deger normalize edilip
kucuk x'e cevriliyor. Dosya yeniden uretildi.

Olcum degismedi: 1673 satirin 1673'unde kesit cikiyor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WQvPu7fT1QvPDBCf8tWdTn
</commit_message>
<xml_diff>
--- a/tests/fixtures/tedarikci_listeleri/Oznur_Kablo_Haziran_2026_PDFten.xlsx
+++ b/tests/fixtures/tedarikci_listeleri/Oznur_Kablo_Haziran_2026_PDFten.xlsx
@@ -11646,7 +11646,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>4x16</t>
         </is>
       </c>
       <c r="E296" t="n">
@@ -11684,7 +11684,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>4x25</t>
         </is>
       </c>
       <c r="E297" t="n">
@@ -11722,7 +11722,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>4x35</t>
         </is>
       </c>
       <c r="E298" t="n">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>4x50</t>
         </is>
       </c>
       <c r="E299" t="n">
@@ -11798,7 +11798,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>4x70</t>
         </is>
       </c>
       <c r="E300" t="n">
@@ -11836,7 +11836,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>4x95</t>
         </is>
       </c>
       <c r="E301" t="n">
@@ -11874,7 +11874,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>4x120</t>
         </is>
       </c>
       <c r="E302" t="n">
@@ -11912,7 +11912,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>4x150</t>
         </is>
       </c>
       <c r="E303" t="n">
@@ -11950,7 +11950,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>185</t>
+          <t>4x185</t>
         </is>
       </c>
       <c r="E304" t="n">
@@ -11988,7 +11988,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>240</t>
+          <t>4x240</t>
         </is>
       </c>
       <c r="E305" t="n">
@@ -12254,7 +12254,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>5x25</t>
         </is>
       </c>
       <c r="E312" t="n">
@@ -12292,7 +12292,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>5x35</t>
         </is>
       </c>
       <c r="E313" t="n">
@@ -12330,7 +12330,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>5x50</t>
         </is>
       </c>
       <c r="E314" t="n">
@@ -12368,7 +12368,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>5x70</t>
         </is>
       </c>
       <c r="E315" t="n">
@@ -12406,7 +12406,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>5x95</t>
         </is>
       </c>
       <c r="E316" t="n">
@@ -12444,7 +12444,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>5x120</t>
         </is>
       </c>
       <c r="E317" t="n">
@@ -12482,7 +12482,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>5x150</t>
         </is>
       </c>
       <c r="E318" t="n">
@@ -12520,7 +12520,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>185</t>
+          <t>5x185</t>
         </is>
       </c>
       <c r="E319" t="n">
@@ -12558,7 +12558,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>240</t>
+          <t>5x240</t>
         </is>
       </c>
       <c r="E320" t="n">
@@ -12976,7 +12976,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>300+150</t>
+          <t>3x300+150</t>
         </is>
       </c>
       <c r="E331" t="n">
@@ -31064,7 +31064,7 @@
       </c>
       <c r="D807" t="inlineStr">
         <is>
-          <t>25+16/16</t>
+          <t>2x25+16/16</t>
         </is>
       </c>
       <c r="E807" t="n">
@@ -31102,7 +31102,7 @@
       </c>
       <c r="D808" t="inlineStr">
         <is>
-          <t>35+16/16</t>
+          <t>2x35+16/16</t>
         </is>
       </c>
       <c r="E808" t="n">
@@ -44326,7 +44326,7 @@
       </c>
       <c r="D1156" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>1x50</t>
         </is>
       </c>
       <c r="E1156" t="n">
@@ -48696,7 +48696,7 @@
       </c>
       <c r="D1271" t="inlineStr">
         <is>
-          <t>16+10</t>
+          <t>3x16+10</t>
         </is>
       </c>
       <c r="E1271" t="n">

</xml_diff>